<commit_message>
Re-collect the 13 Sep Google News screen and confirm it is unchanged.
The 19:43 MSK RSS pass matches the 19:39 snapshot card-for-card. Publisher URLs are now copied from earlier screens before reports are written, and the Excel pack compares this run with 23 Aug plus a same-day control workbook.

Co-authored-by: Ilya Rost <jaguarcatcat@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/sravnenie_vydachi.xlsx
+++ b/output/sravnenie_vydachi.xlsx
@@ -546,7 +546,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-13T19:39:11+03:00</t>
+          <t>2026-09-13T19:43:10+03:00</t>
         </is>
       </c>
     </row>
@@ -669,9 +669,9 @@
     <col width="58" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
     <col width="31" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -703,17 +703,17 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Позиция: 17 августа</t>
+          <t>Позиция: 17 авг</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Позиция: 23 августа</t>
+          <t>Позиция: 23 авг</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Позиция: 13 сентября</t>
+          <t>Позиция: 13 сен 19:43</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -15413,7 +15413,7 @@
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>2026-08-23T19:33:41+03:00 → 2026-09-13T19:39:11+03:00</t>
+          <t>2026-08-23T19:33:41+03:00 → 2026-09-13T19:43:10+03:00</t>
         </is>
       </c>
     </row>

</xml_diff>